<commit_message>
test: add UI regression and consolidate testing evidence
</commit_message>
<xml_diff>
--- a/test-functional/Litemall功能测试用例.xlsx
+++ b/test-functional/Litemall功能测试用例.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="用户端用例" sheetId="1" r:id="Rea053eed5942486b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="管理端用例" sheetId="2" r:id="R14e1f9edb13b4b8a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="跨端闭环" sheetId="3" r:id="Rb26703545e164fc9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="用户端用例" sheetId="1" r:id="R54fa1e31c50047dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="管理端用例" sheetId="2" r:id="R47915294d88d4e82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="跨端闭环" sheetId="3" r:id="R6506d2492c22443d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1065,7 +1065,7 @@
         <x:v>返回匹配商品；关键词、总数和分页正确</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="48" customHeight="1">
+    <x:row r="11" ht="24" hidden="0" customHeight="1">
       <x:c r="A11" s="50" t="str">
         <x:v>U-SEARCH-002</x:v>
       </x:c>
@@ -1086,13 +1086,13 @@
 2. 观察页面提示、接口响应及业务状态</x:v>
       </x:c>
       <x:c r="G11" s="51" t="str">
-        <x:v>存在词：宠物；不存在词：zz_no_goods_20261012；特殊字符：%_'"&lt;&gt;；结果数大于每页条数的数据集</x:v>
+        <x:v>不存在关键词=zz_no_goods_20261027；使用同一关键词查接口确认结果集合为空</x:v>
       </x:c>
       <x:c r="H11" s="53" t="str">
         <x:v>返回空列表和合理空态；不报系统错误</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="48" customHeight="1">
+    <x:row r="12" ht="24" hidden="0" customHeight="1">
       <x:c r="A12" s="50" t="str">
         <x:v>U-SEARCH-003</x:v>
       </x:c>
@@ -1113,7 +1113,7 @@
 2. 观察页面提示、接口响应及业务状态</x:v>
       </x:c>
       <x:c r="G12" s="51" t="str">
-        <x:v>存在词：宠物；不存在词：zz_no_goods_20261012；特殊字符：%_'"&lt;&gt;；结果数大于每页条数的数据集</x:v>
+        <x:v>基准关键词=宠物；对比输入="  宠物  "；其余筛选条件保持相同</x:v>
       </x:c>
       <x:c r="H12" s="53" t="str">
         <x:v>按产品约定去空格或给出提示；不能出现不可解释的不同结果</x:v>
@@ -1173,7 +1173,7 @@
         <x:v>请求被安全处理；无 SQL/HTML 异常；结果或提示合理</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="48" customHeight="1">
+    <x:row r="15" ht="24" hidden="0" customHeight="1">
       <x:c r="A15" s="50" t="str">
         <x:v>U-SEARCH-006</x:v>
       </x:c>
@@ -1181,7 +1181,7 @@
         <x:v>搜索联想</x:v>
       </x:c>
       <x:c r="C15" s="51" t="str">
-        <x:v>H5/小程序-搜索</x:v>
+        <x:v>小程序-搜索</x:v>
       </x:c>
       <x:c r="D15" s="52" t="str">
         <x:v>P1</x:v>
@@ -1254,7 +1254,7 @@
         <x:v>历史清空；刷新后仍为空；不影响热门词</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="48" customHeight="1">
+    <x:row r="18" ht="24" hidden="0" customHeight="1">
       <x:c r="A18" s="50" t="str">
         <x:v>U-SEARCH-009</x:v>
       </x:c>
@@ -1262,7 +1262,7 @@
         <x:v>商品排序</x:v>
       </x:c>
       <x:c r="C18" s="51" t="str">
-        <x:v>H5/小程序-搜索</x:v>
+        <x:v>小程序-搜索</x:v>
       </x:c>
       <x:c r="D18" s="52" t="str">
         <x:v>P2</x:v>
@@ -1308,7 +1308,7 @@
         <x:v>无重复/遗漏；最后一页后不继续发无效请求</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="48" customHeight="1">
+    <x:row r="20" ht="48" hidden="0" customHeight="1">
       <x:c r="A20" s="50" t="str">
         <x:v>U-AUTH-001</x:v>
       </x:c>
@@ -1325,17 +1325,19 @@
         <x:v>Litemall后端和MySQL可访问；有效账号</x:v>
       </x:c>
       <x:c r="F20" s="51" t="str">
-        <x:v>1. 输入正确账号密码登录
-2. 观察页面提示、接口响应及业务状态</x:v>
+        <x:v>1. 打开H5登录页或小程序账号登录页
+2. 输入本地测试账号user123/user123并点击登录
+3. 检查个人中心用户名与登录响应Token
+4. 刷新后再次访问个人中心，核对登录态</x:v>
       </x:c>
       <x:c r="G20" s="51" t="str">
-        <x:v>有效账号test123/正确密码；错误密码Wrong123；不存在账号no_user_20261012；无效token=invalid-token</x:v>
+        <x:v>本地有效账号user123/user123；错误密码Wrong123；不存在账号no_user_20261012；无效token=invalid-token</x:v>
       </x:c>
       <x:c r="H20" s="53" t="str">
         <x:v>HTTP 与业务均成功；获得 token；进入用户页；刷新后登录态符合产品约定</x:v>
       </x:c>
     </x:row>
-    <x:row r="21" ht="48" customHeight="1">
+    <x:row r="21" ht="48" hidden="0" customHeight="1">
       <x:c r="A21" s="50" t="str">
         <x:v>U-AUTH-002</x:v>
       </x:c>
@@ -1352,17 +1354,19 @@
         <x:v>Litemall后端和MySQL可访问；有效账号、错误密码</x:v>
       </x:c>
       <x:c r="F21" s="51" t="str">
-        <x:v>1. 登录
-2. 观察页面提示、接口响应及业务状态</x:v>
+        <x:v>1. 打开账号登录页
+2. 输入user123及错误密码Wrong123并提交
+3. 核对错误提示、当前页面和响应
+4. 尝试访问受保护资源，确认未建立有效登录态</x:v>
       </x:c>
       <x:c r="G21" s="51" t="str">
-        <x:v>有效账号test123/正确密码；错误密码Wrong123；不存在账号no_user_20261012；无效token=invalid-token</x:v>
+        <x:v>本地有效账号user123/user123；错误密码Wrong123；不存在账号no_user_20261012；无效token=invalid-token</x:v>
       </x:c>
       <x:c r="H21" s="53" t="str">
         <x:v>业务失败并提示账号或密码错误；不返回 token；不进入登录态</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" ht="48" customHeight="1">
+    <x:row r="22" ht="24" hidden="0" customHeight="1">
       <x:c r="A22" s="50" t="str">
         <x:v>U-AUTH-003</x:v>
       </x:c>
@@ -1383,13 +1387,13 @@
 2. 观察页面提示、接口响应及业务状态</x:v>
       </x:c>
       <x:c r="G22" s="51" t="str">
-        <x:v>有效账号test123/正确密码；错误密码Wrong123；不存在账号no_user_20261012；无效token=invalid-token</x:v>
+        <x:v>本地有效账号user123/user123；错误密码Wrong123；不存在账号no_user_20261012；无效token=invalid-token</x:v>
       </x:c>
       <x:c r="H22" s="53" t="str">
         <x:v>明确失败；不泄露用户是否存在等敏感细节；无 token</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" ht="48" customHeight="1">
+    <x:row r="23" ht="24" hidden="0" customHeight="1">
       <x:c r="A23" s="50" t="str">
         <x:v>U-AUTH-004</x:v>
       </x:c>
@@ -1410,13 +1414,13 @@
 2. 观察页面提示、接口响应及业务状态</x:v>
       </x:c>
       <x:c r="G23" s="51" t="str">
-        <x:v>有效账号test123/正确密码；错误密码Wrong123；不存在账号no_user_20261012；无效token=invalid-token</x:v>
+        <x:v>本地有效账号user123/user123；错误密码Wrong123；不存在账号no_user_20261012；无效token=invalid-token</x:v>
       </x:c>
       <x:c r="H23" s="53" t="str">
         <x:v>前端校验或后端返回参数错误；不发起成功登录</x:v>
       </x:c>
     </x:row>
-    <x:row r="24" ht="48" customHeight="1">
+    <x:row r="24" ht="24" hidden="0" customHeight="1">
       <x:c r="A24" s="50" t="str">
         <x:v>U-AUTH-005</x:v>
       </x:c>
@@ -1437,13 +1441,13 @@
 2. 观察页面提示、接口响应及业务状态</x:v>
       </x:c>
       <x:c r="G24" s="51" t="str">
-        <x:v>有效账号test123/正确密码；错误密码Wrong123；不存在账号no_user_20261012；无效token=invalid-token</x:v>
+        <x:v>本地有效账号user123/user123；错误密码Wrong123；不存在账号no_user_20261012；无效token=invalid-token</x:v>
       </x:c>
       <x:c r="H24" s="53" t="str">
         <x:v>输入不被截断或转义错误；结果符合账号真实密码</x:v>
       </x:c>
     </x:row>
-    <x:row r="25" ht="48" customHeight="1">
+    <x:row r="25" ht="24" hidden="0" customHeight="1">
       <x:c r="A25" s="50" t="str">
         <x:v>U-AUTH-006</x:v>
       </x:c>
@@ -1464,13 +1468,13 @@
 2. 观察页面提示、接口响应及业务状态</x:v>
       </x:c>
       <x:c r="G25" s="51" t="str">
-        <x:v>有效账号test123/正确密码；错误密码Wrong123；不存在账号no_user_20261012；无效token=invalid-token</x:v>
+        <x:v>本地有效账号user123/user123；错误密码Wrong123；不存在账号no_user_20261012；无效token=invalid-token</x:v>
       </x:c>
       <x:c r="H25" s="53" t="str">
         <x:v>跳转登录或返回未登录；不得泄露用户数据</x:v>
       </x:c>
     </x:row>
-    <x:row r="26" ht="48" customHeight="1">
+    <x:row r="26" ht="24" hidden="0" customHeight="1">
       <x:c r="A26" s="50" t="str">
         <x:v>U-AUTH-007</x:v>
       </x:c>
@@ -1491,13 +1495,13 @@
 2. 观察页面提示、接口响应及业务状态</x:v>
       </x:c>
       <x:c r="G26" s="51" t="str">
-        <x:v>有效账号test123/正确密码；错误密码Wrong123；不存在账号no_user_20261012；无效token=invalid-token</x:v>
+        <x:v>本地有效账号user123/user123；错误密码Wrong123；不存在账号no_user_20261012；无效token=invalid-token</x:v>
       </x:c>
       <x:c r="H26" s="53" t="str">
         <x:v>被拒绝并清理失效登录态；不得返回原用户数据</x:v>
       </x:c>
     </x:row>
-    <x:row r="27" ht="48" customHeight="1">
+    <x:row r="27" ht="24" hidden="0" customHeight="1">
       <x:c r="A27" s="50" t="str">
         <x:v>U-AUTH-008</x:v>
       </x:c>
@@ -1518,13 +1522,13 @@
 2. 观察页面提示、接口响应及业务状态</x:v>
       </x:c>
       <x:c r="G27" s="51" t="str">
-        <x:v>有效账号test123/正确密码；错误密码Wrong123；不存在账号no_user_20261012；无效token=invalid-token</x:v>
+        <x:v>本地有效账号user123/user123；错误密码Wrong123；不存在账号no_user_20261012；无效token=invalid-token</x:v>
       </x:c>
       <x:c r="H27" s="53" t="str">
         <x:v>token/会话失效；返回登录页；浏览器返回不能恢复敏感数据</x:v>
       </x:c>
     </x:row>
-    <x:row r="28" ht="48" customHeight="1">
+    <x:row r="28" ht="24" hidden="0" customHeight="1">
       <x:c r="A28" s="50" t="str">
         <x:v>U-AUTH-009</x:v>
       </x:c>
@@ -1545,13 +1549,13 @@
 2. 观察页面提示、接口响应及业务状态</x:v>
       </x:c>
       <x:c r="G28" s="51" t="str">
-        <x:v>有效账号test123/正确密码；错误密码Wrong123；不存在账号no_user_20261012；无效token=invalid-token</x:v>
+        <x:v>本地有效账号user123/user123；错误密码Wrong123；不存在账号no_user_20261012；无效token=invalid-token</x:v>
       </x:c>
       <x:c r="H28" s="53" t="str">
         <x:v>注册成功并按约定登录；用户记录唯一；密码安全存储</x:v>
       </x:c>
     </x:row>
-    <x:row r="29" ht="48" customHeight="1">
+    <x:row r="29" ht="24" hidden="0" customHeight="1">
       <x:c r="A29" s="50" t="str">
         <x:v>U-AUTH-010</x:v>
       </x:c>
@@ -1572,13 +1576,13 @@
 2. 观察页面提示、接口响应及业务状态</x:v>
       </x:c>
       <x:c r="G29" s="51" t="str">
-        <x:v>有效账号test123/正确密码；错误密码Wrong123；不存在账号no_user_20261012；无效token=invalid-token</x:v>
+        <x:v>本地有效账号user123/user123；错误密码Wrong123；不存在账号no_user_20261012；无效token=invalid-token</x:v>
       </x:c>
       <x:c r="H29" s="53" t="str">
         <x:v>明确提示已存在；不新增重复用户</x:v>
       </x:c>
     </x:row>
-    <x:row r="30" ht="48" customHeight="1">
+    <x:row r="30" ht="24" hidden="0" customHeight="1">
       <x:c r="A30" s="50" t="str">
         <x:v>U-AUTH-011</x:v>
       </x:c>
@@ -1599,13 +1603,13 @@
 2. 观察页面提示、接口响应及业务状态</x:v>
       </x:c>
       <x:c r="G30" s="51" t="str">
-        <x:v>有效账号test123/正确密码；错误密码Wrong123；不存在账号no_user_20261012；无效token=invalid-token</x:v>
+        <x:v>本地有效账号user123/user123；错误密码Wrong123；不存在账号no_user_20261012；无效token=invalid-token</x:v>
       </x:c>
       <x:c r="H30" s="53" t="str">
         <x:v>均被拒绝；验证码一次性和有效期规则正确</x:v>
       </x:c>
     </x:row>
-    <x:row r="31" ht="48" customHeight="1">
+    <x:row r="31" ht="24" hidden="0" customHeight="1">
       <x:c r="A31" s="50" t="str">
         <x:v>U-AUTH-012</x:v>
       </x:c>
@@ -1626,13 +1630,13 @@
 2. 观察页面提示、接口响应及业务状态</x:v>
       </x:c>
       <x:c r="G31" s="51" t="str">
-        <x:v>有效账号test123/正确密码；错误密码Wrong123；不存在账号no_user_20261012；无效token=invalid-token</x:v>
+        <x:v>本地有效账号user123/user123；错误密码Wrong123；不存在账号no_user_20261012；无效token=invalid-token</x:v>
       </x:c>
       <x:c r="H31" s="53" t="str">
         <x:v>超频被限制且提示明确；未产生大量短信任务</x:v>
       </x:c>
     </x:row>
-    <x:row r="32" ht="48" customHeight="1">
+    <x:row r="32" ht="24" hidden="0" customHeight="1">
       <x:c r="A32" s="50" t="str">
         <x:v>U-AUTH-013</x:v>
       </x:c>
@@ -1653,13 +1657,13 @@
 2. 观察页面提示、接口响应及业务状态</x:v>
       </x:c>
       <x:c r="G32" s="51" t="str">
-        <x:v>有效账号test123/正确密码；错误密码Wrong123；不存在账号no_user_20261012；无效token=invalid-token</x:v>
+        <x:v>本地有效账号user123/user123；错误密码Wrong123；不存在账号no_user_20261012；无效token=invalid-token</x:v>
       </x:c>
       <x:c r="H32" s="53" t="str">
         <x:v>重置成功；旧密码失效；新密码可登录</x:v>
       </x:c>
     </x:row>
-    <x:row r="33" ht="48" customHeight="1">
+    <x:row r="33" ht="24" hidden="0" customHeight="1">
       <x:c r="A33" s="50" t="str">
         <x:v>U-AUTH-014</x:v>
       </x:c>
@@ -1680,13 +1684,13 @@
 2. 观察页面提示、接口响应及业务状态</x:v>
       </x:c>
       <x:c r="G33" s="51" t="str">
-        <x:v>有效账号test123/正确密码；错误密码Wrong123；不存在账号no_user_20261012；无效token=invalid-token</x:v>
+        <x:v>本地有效账号user123/user123；错误密码Wrong123；不存在账号no_user_20261012；无效token=invalid-token</x:v>
       </x:c>
       <x:c r="H33" s="53" t="str">
         <x:v>更新成功；重新登录仍保留；其他用户数据不变</x:v>
       </x:c>
     </x:row>
-    <x:row r="34" ht="48" customHeight="1">
+    <x:row r="34" ht="24" hidden="0" customHeight="1">
       <x:c r="A34" s="50" t="str">
         <x:v>U-AUTH-015</x:v>
       </x:c>
@@ -1707,13 +1711,13 @@
 2. 观察页面提示、接口响应及业务状态</x:v>
       </x:c>
       <x:c r="G34" s="51" t="str">
-        <x:v>有效账号test123/正确密码；错误密码Wrong123；不存在账号no_user_20261012；无效token=invalid-token</x:v>
+        <x:v>本地有效账号user123/user123；错误密码Wrong123；不存在账号no_user_20261012；无效token=invalid-token</x:v>
       </x:c>
       <x:c r="H34" s="53" t="str">
         <x:v>绑定成功且唯一；错误验证码/已占用手机号被拒绝</x:v>
       </x:c>
     </x:row>
-    <x:row r="35" ht="48" customHeight="1">
+    <x:row r="35" ht="24" hidden="0" customHeight="1">
       <x:c r="A35" s="50" t="str">
         <x:v>U-AUTH-016</x:v>
       </x:c>
@@ -1734,13 +1738,13 @@
 2. 观察页面提示、接口响应及业务状态</x:v>
       </x:c>
       <x:c r="G35" s="51" t="str">
-        <x:v>有效账号test123/正确密码；错误密码Wrong123；不存在账号no_user_20261012；无效token=invalid-token</x:v>
+        <x:v>本地有效账号user123/user123；错误密码Wrong123；不存在账号no_user_20261012；无效token=invalid-token</x:v>
       </x:c>
       <x:c r="H35" s="53" t="str">
         <x:v>code 换取会话成功；首次创建/再次复用同一用户；不重复建号</x:v>
       </x:c>
     </x:row>
-    <x:row r="36" ht="48" customHeight="1">
+    <x:row r="36" ht="24" hidden="0" customHeight="1">
       <x:c r="A36" s="50" t="str">
         <x:v>U-AUTH-017</x:v>
       </x:c>
@@ -1761,13 +1765,13 @@
 2. 观察页面提示、接口响应及业务状态</x:v>
       </x:c>
       <x:c r="G36" s="51" t="str">
-        <x:v>有效账号test123/正确密码；错误密码Wrong123；不存在账号no_user_20261012；无效token=invalid-token</x:v>
+        <x:v>本地有效账号user123/user123；错误密码Wrong123；不存在账号no_user_20261012；无效token=invalid-token</x:v>
       </x:c>
       <x:c r="H36" s="53" t="str">
         <x:v>有明确提示和可重试入口；页面不死循环</x:v>
       </x:c>
     </x:row>
-    <x:row r="37" ht="48" customHeight="1">
+    <x:row r="37" ht="24" hidden="0" customHeight="1">
       <x:c r="A37" s="50" t="str">
         <x:v>U-AUTH-018</x:v>
       </x:c>
@@ -1788,7 +1792,7 @@
 2. 观察页面提示、接口响应及业务状态</x:v>
       </x:c>
       <x:c r="G37" s="51" t="str">
-        <x:v>有效账号test123/正确密码；错误密码Wrong123；不存在账号no_user_20261012；无效token=invalid-token</x:v>
+        <x:v>本地有效账号user123/user123；错误密码Wrong123；不存在账号no_user_20261012；无效token=invalid-token</x:v>
       </x:c>
       <x:c r="H37" s="53" t="str">
         <x:v>返回原目标页或合理默认页；关键上下文按约定保留</x:v>
@@ -1821,7 +1825,7 @@
         <x:v>基本信息、图片、规格、价格、库存、属性、评价、关联商品正确</x:v>
       </x:c>
     </x:row>
-    <x:row r="39" ht="48" customHeight="1">
+    <x:row r="39" ht="48" hidden="0" customHeight="1">
       <x:c r="A39" s="50" t="str">
         <x:v>U-GOODS-002</x:v>
       </x:c>
@@ -1838,8 +1842,10 @@
         <x:v>Litemall后端和MySQL可访问；</x:v>
       </x:c>
       <x:c r="F39" s="51" t="str">
-        <x:v>1. 打开详情
-2. 观察页面提示、接口响应及业务状态</x:v>
+        <x:v>1. 使用不存在商品ID=999999999打开商品详情
+2. 在接口工具中查询同一ID并记录响应
+3. 核对商品不存在业务提示
+4. 检查同一时间窗服务日志是否出现异常</x:v>
       </x:c>
       <x:c r="G39" s="51" t="str">
         <x:v>有效商品ID=1110016；不存在ID=999999999；上架/下架商品各1个；多规格、零库存SKU各1个</x:v>
@@ -2307,7 +2313,7 @@
         <x:v>被拒绝；人数和状态不变</x:v>
       </x:c>
     </x:row>
-    <x:row r="57" ht="48" customHeight="1">
+    <x:row r="57" ht="48" hidden="0" customHeight="1">
       <x:c r="A57" s="50" t="str">
         <x:v>U-CART-001</x:v>
       </x:c>
@@ -2324,8 +2330,10 @@
         <x:v>Litemall后端和MySQL可访问；已登录、可售 SKU、库存充足</x:v>
       </x:c>
       <x:c r="F57" s="51" t="str">
-        <x:v>1. 选择规格和数量加购
-2. 观察页面提示、接口响应及业务状态</x:v>
+        <x:v>1. 登录后打开有效商品详情
+2. 选择完整规格及数量1，点击加入购物车
+3. 打开购物车核对名称、规格、数量和价格
+4. 查询购物车接口，核对同一SKU记录及角标数量</x:v>
       </x:c>
       <x:c r="G57" s="51" t="str">
         <x:v>用户A、用户B；商品ID=1110016；有效productId=150；库存N；数量0、1、N、N+1</x:v>
@@ -2415,7 +2423,7 @@
         <x:v>被拒绝或限制为 N；数据库数量不超过库存</x:v>
       </x:c>
     </x:row>
-    <x:row r="61" ht="48" customHeight="1">
+    <x:row r="61" ht="72" hidden="0" customHeight="1">
       <x:c r="A61" s="50" t="str">
         <x:v>U-CART-005</x:v>
       </x:c>
@@ -2432,8 +2440,10 @@
         <x:v>Litemall后端和MySQL可访问；购物车已有商品</x:v>
       </x:c>
       <x:c r="F61" s="51" t="str">
-        <x:v>1. 改为 0、1、N、N+1、负数、非整数
-2. 观察页面提示、接口响应及业务状态</x:v>
+        <x:v>1. 准备库存为N且已加入购物车的商品
+2. 分别修改数量为0、1、N、N+1、负数和非整数
+3. 对每组输入核对页面提示、合计与接口业务结果
+4. 重新查询购物车，确认合法值保存、非法值未落库；恢复原数量</x:v>
       </x:c>
       <x:c r="G61" s="51" t="str">
         <x:v>用户A、用户B；商品ID=1110016；有效productId=150；库存N；数量0、1、N、N+1</x:v>
@@ -2685,7 +2695,7 @@
         <x:v>被拒绝；用户券数量不增加</x:v>
       </x:c>
     </x:row>
-    <x:row r="71" ht="48" customHeight="1">
+    <x:row r="71" ht="24" hidden="0" customHeight="1">
       <x:c r="A71" s="50" t="str">
         <x:v>U-COUPON-003</x:v>
       </x:c>
@@ -2699,7 +2709,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="E71" s="51" t="str">
-        <x:v>Litemall后端和MySQL可访问；正确未</x:v>
+        <x:v>Litemall后端和MySQL可访问；用户已登录；准备正确、有效且未被该用户兑换的兑换码</x:v>
       </x:c>
       <x:c r="F71" s="51" t="str">
         <x:v>1. 兑换
@@ -2847,7 +2857,7 @@
         <x:v>券恢复可用；订单与券状态一致；不可重复释放</x:v>
       </x:c>
     </x:row>
-    <x:row r="77" ht="48" customHeight="1">
+    <x:row r="77" ht="48" hidden="0" customHeight="1">
       <x:c r="A77" s="50" t="str">
         <x:v>U-ADDR-001</x:v>
       </x:c>
@@ -2864,8 +2874,10 @@
         <x:v>Litemall后端和MySQL可访问；已登录</x:v>
       </x:c>
       <x:c r="F77" s="51" t="str">
-        <x:v>1. 填写完整省市区、姓名、手机号、地址并保存
-2. 观察页面提示、接口响应及业务状态</x:v>
+        <x:v>1. 登录用户A并进入新增收货地址页
+2. 填写完整姓名、手机号、省市区和详细地址后保存
+3. 从列表打开新地址详情，逐字段核对
+4. 在结算页选择该地址，核对显示；完成后清理临时地址</x:v>
       </x:c>
       <x:c r="G77" s="51" t="str">
         <x:v>用户A/B；姓名=测试用户；手机号=13800138000；省市区及详细地址；他人地址ID 1个</x:v>
@@ -3090,7 +3102,7 @@
         <x:v>商品、数量、价格、运费、优惠券候选、应付金额正确</x:v>
       </x:c>
     </x:row>
-    <x:row r="86" ht="48" customHeight="1">
+    <x:row r="86" ht="190" hidden="0" customHeight="1">
       <x:c r="A86" s="50" t="str">
         <x:v>U-ORDER-002</x:v>
       </x:c>
@@ -3107,8 +3119,11 @@
         <x:v>Litemall后端和MySQL可访问；库存充足、数据有效</x:v>
       </x:c>
       <x:c r="F86" s="51" t="str">
-        <x:v>1. 提交一次
-2. 观察页面提示、接口响应及业务状态</x:v>
+        <x:v>1. 登录并准备库存充足的商品、购物车和本人地址
+2. 进入结算，核对商品、数量、运费与应付金额
+3. 仅点击一次提交并记录返回的orderId
+4. 查看待付款页面及订单详情，核对金额、商品和状态
+5. 查库核对订单主表、明细、购物车与库存；取消并清理测试订单</x:v>
       </x:c>
       <x:c r="G86" s="51" t="str">
         <x:v>用户A/B；有效商品与SKU；地址ID；可用/不可用优惠券；库存N；订单金额与运费配置</x:v>
@@ -3252,7 +3267,7 @@
         <x:v>至多一个成功；库存不为负；失败方有明确提示</x:v>
       </x:c>
     </x:row>
-    <x:row r="92" ht="48" customHeight="1">
+    <x:row r="92" ht="190" hidden="0" customHeight="1">
       <x:c r="A92" s="50" t="str">
         <x:v>U-ORDER-008</x:v>
       </x:c>
@@ -3269,14 +3284,17 @@
         <x:v>Litemall后端和MySQL可访问；合法结算数据</x:v>
       </x:c>
       <x:c r="F92" s="51" t="str">
-        <x:v>1. 双击、重放相同请求
-2. 观察页面提示、接口响应及业务状态</x:v>
+        <x:v>1. 准备合法购物车及本人地址，记录cartId和SKU原库存
+2. 提交一次订单，保存orderId
+3. 保持同一用户、cartId和业务参数，再次发送相同请求
+4. 核对第二次响应、订单数与库存，确认没有新增重复订单
+5. 保存两次请求响应与数据库证据，清理本次生成订单并恢复库存</x:v>
       </x:c>
       <x:c r="G92" s="51" t="str">
         <x:v>用户A/B；有效商品与SKU；地址ID；可用/不可用优惠券；库存N；订单金额与运费配置</x:v>
       </x:c>
       <x:c r="H92" s="53" t="str">
-        <x:v>不产生不可解释的重复订单或重复扣库存；若业务允许多单，应有明确幂等边界</x:v>
+        <x:v>相同cartId对应的同一提交操作仅创建一个订单、仅扣减一次库存；重放请求应被拒绝或返回首次处理结果，不得生成新的订单ID</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="48" customHeight="1">
@@ -3711,7 +3729,7 @@
         <x:v>评价成功；订单明细评价标志更新；商品评价可见</x:v>
       </x:c>
     </x:row>
-    <x:row r="109" ht="48" customHeight="1">
+    <x:row r="109" ht="36" hidden="0" customHeight="1">
       <x:c r="A109" s="50" t="str">
         <x:v>U-ORDER-025</x:v>
       </x:c>
@@ -3725,7 +3743,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="E109" s="51" t="str">
-        <x:v>Litemall后端和MySQL可访问；已评价或</x:v>
+        <x:v>Litemall后端和MySQL可访问；分别准备当前用户已评价的订单商品，以及属于用户A、尚未评价的订单商品；用户B已登录</x:v>
       </x:c>
       <x:c r="F109" s="51" t="str">
         <x:v>1. 提交评价
@@ -3819,7 +3837,7 @@
         <x:v>按规则校验；合法边界金额精度正确</x:v>
       </x:c>
     </x:row>
-    <x:row r="113" ht="48" customHeight="1">
+    <x:row r="113" ht="24" hidden="0" customHeight="1">
       <x:c r="A113" s="50" t="str">
         <x:v>U-AFTER-004</x:v>
       </x:c>
@@ -3833,7 +3851,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="E113" s="51" t="str">
-        <x:v>Litemall后端和MySQL可访问；B</x:v>
+        <x:v>Litemall后端和MySQL可访问；用户A有满足售后条件的订单；用户B已登录并取得该订单ID</x:v>
       </x:c>
       <x:c r="F113" s="51" t="str">
         <x:v>1. 提交
@@ -4520,7 +4538,7 @@
         <x:v>预期结果</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="48" customHeight="1">
+    <x:row r="2" ht="36" hidden="0" customHeight="1">
       <x:c r="A2" s="50" t="str">
         <x:v>A-AUTH-001</x:v>
       </x:c>
@@ -4541,13 +4559,13 @@
 2. 观察页面提示、接口响应及业务状态</x:v>
       </x:c>
       <x:c r="G2" s="51" t="str">
-        <x:v>有效账号test123/正确密码；错误密码Wrong123；不存在账号no_user_20261012；无效token=invalid-token</x:v>
+        <x:v>有效管理员admin及本机配置中的管理端密码；错误密码Wrong123；不存在管理员no_admin_20261027；普通角色账号；无效管理端Token</x:v>
       </x:c>
       <x:c r="H2" s="53" t="str">
         <x:v>登录成功；返回 token、角色和权限；进入工作台</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="48" customHeight="1">
+    <x:row r="3" ht="36" hidden="0" customHeight="1">
       <x:c r="A3" s="50" t="str">
         <x:v>A-AUTH-002</x:v>
       </x:c>
@@ -4568,13 +4586,13 @@
 2. 观察页面提示、接口响应及业务状态</x:v>
       </x:c>
       <x:c r="G3" s="51" t="str">
-        <x:v>有效账号test123/正确密码；错误密码Wrong123；不存在账号no_user_20261012；无效token=invalid-token</x:v>
+        <x:v>有效管理员admin及本机配置中的管理端密码；错误密码Wrong123；不存在管理员no_admin_20261027；普通角色账号；无效管理端Token</x:v>
       </x:c>
       <x:c r="H3" s="53" t="str">
         <x:v>明确失败；无 token；不泄露敏感信息</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="48" customHeight="1">
+    <x:row r="4" ht="36" hidden="0" customHeight="1">
       <x:c r="A4" s="50" t="str">
         <x:v>A-AUTH-003</x:v>
       </x:c>
@@ -4595,13 +4613,13 @@
 2. 观察页面提示、接口响应及业务状态</x:v>
       </x:c>
       <x:c r="G4" s="51" t="str">
-        <x:v>有效账号test123/正确密码；错误密码Wrong123；不存在账号no_user_20261012；无效token=invalid-token</x:v>
+        <x:v>有效管理员admin及本机配置中的管理端密码；错误密码Wrong123；不存在管理员no_admin_20261027；普通角色账号；无效管理端Token</x:v>
       </x:c>
       <x:c r="H4" s="53" t="str">
         <x:v>均被拒绝；刷新后旧验证码不可继续使用</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="48" customHeight="1">
+    <x:row r="5" ht="36" hidden="0" customHeight="1">
       <x:c r="A5" s="50" t="str">
         <x:v>A-AUTH-004</x:v>
       </x:c>
@@ -4622,13 +4640,13 @@
 2. 观察页面提示、接口响应及业务状态</x:v>
       </x:c>
       <x:c r="G5" s="51" t="str">
-        <x:v>有效账号test123/正确密码；错误密码Wrong123；不存在账号no_user_20261012；无效token=invalid-token</x:v>
+        <x:v>有效管理员admin及本机配置中的管理端密码；错误密码Wrong123；不存在管理员no_admin_20261027；普通角色账号；无效管理端Token</x:v>
       </x:c>
       <x:c r="H5" s="53" t="str">
         <x:v>按项目规则记录/限制；服务不崩溃；日志可追踪</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="48" customHeight="1">
+    <x:row r="6" ht="36" hidden="0" customHeight="1">
       <x:c r="A6" s="50" t="str">
         <x:v>A-AUTH-005</x:v>
       </x:c>
@@ -4649,13 +4667,13 @@
 2. 观察页面提示、接口响应及业务状态</x:v>
       </x:c>
       <x:c r="G6" s="51" t="str">
-        <x:v>有效账号test123/正确密码；错误密码Wrong123；不存在账号no_user_20261012；无效token=invalid-token</x:v>
+        <x:v>有效管理员admin及本机配置中的管理端密码；错误密码Wrong123；不存在管理员no_admin_20261027；普通角色账号；无效管理端Token</x:v>
       </x:c>
       <x:c r="H6" s="53" t="str">
         <x:v>跳转登录或 401；不得返回后台数据</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="48" customHeight="1">
+    <x:row r="7" ht="36" hidden="0" customHeight="1">
       <x:c r="A7" s="50" t="str">
         <x:v>A-AUTH-006</x:v>
       </x:c>
@@ -4676,13 +4694,13 @@
 2. 观察页面提示、接口响应及业务状态</x:v>
       </x:c>
       <x:c r="G7" s="51" t="str">
-        <x:v>有效账号test123/正确密码；错误密码Wrong123；不存在账号no_user_20261012；无效token=invalid-token</x:v>
+        <x:v>有效管理员admin及本机配置中的管理端密码；错误密码Wrong123；不存在管理员no_admin_20261027；普通角色账号；无效管理端Token</x:v>
       </x:c>
       <x:c r="H7" s="53" t="str">
         <x:v>菜单不可见且服务端拒绝；不能仅靠前端隐藏</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="48" customHeight="1">
+    <x:row r="8" ht="36" hidden="0" customHeight="1">
       <x:c r="A8" s="50" t="str">
         <x:v>A-AUTH-007</x:v>
       </x:c>
@@ -4703,13 +4721,13 @@
 2. 观察页面提示、接口响应及业务状态</x:v>
       </x:c>
       <x:c r="G8" s="51" t="str">
-        <x:v>有效账号test123/正确密码；错误密码Wrong123；不存在账号no_user_20261012；无效token=invalid-token</x:v>
+        <x:v>有效管理员admin及本机配置中的管理端密码；错误密码Wrong123；不存在管理员no_admin_20261027；普通角色账号；无效管理端Token</x:v>
       </x:c>
       <x:c r="H8" s="53" t="str">
         <x:v>会话失效；旧 token 不能继续访问</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="48" customHeight="1">
+    <x:row r="9" ht="36" hidden="0" customHeight="1">
       <x:c r="A9" s="50" t="str">
         <x:v>A-AUTH-008</x:v>
       </x:c>
@@ -4730,13 +4748,13 @@
 2. 观察页面提示、接口响应及业务状态</x:v>
       </x:c>
       <x:c r="G9" s="51" t="str">
-        <x:v>有效账号test123/正确密码；错误密码Wrong123；不存在账号no_user_20261012；无效token=invalid-token</x:v>
+        <x:v>有效管理员admin及本机配置中的管理端密码；错误密码Wrong123；不存在管理员no_admin_20261027；普通角色账号；无效管理端Token</x:v>
       </x:c>
       <x:c r="H9" s="53" t="str">
         <x:v>修改成功；旧密码失效；新密码登录成功</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="48" customHeight="1">
+    <x:row r="10" ht="36" hidden="0" customHeight="1">
       <x:c r="A10" s="50" t="str">
         <x:v>A-AUTH-009</x:v>
       </x:c>
@@ -4757,7 +4775,7 @@
 2. 观察页面提示、接口响应及业务状态</x:v>
       </x:c>
       <x:c r="G10" s="51" t="str">
-        <x:v>有效账号test123/正确密码；错误密码Wrong123；不存在账号no_user_20261012；无效token=invalid-token</x:v>
+        <x:v>有效管理员admin及本机配置中的管理端密码；错误密码Wrong123；不存在管理员no_admin_20261027；普通角色账号；无效管理端Token</x:v>
       </x:c>
       <x:c r="H10" s="53" t="str">
         <x:v>被拒绝；原密码仍有效</x:v>
@@ -7087,7 +7105,7 @@
         <x:v>不超卖；库存扣减准确；取消后按规则恢复且只恢复一次</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="48" customHeight="1">
+    <x:row r="6" ht="24" hidden="0" customHeight="1">
       <x:c r="A6" s="50" t="str">
         <x:v>E2E-005</x:v>
       </x:c>
@@ -7108,7 +7126,7 @@
 2. 观察页面提示、接口响应及业务状态</x:v>
       </x:c>
       <x:c r="G6" s="51" t="str">
-        <x:v>管理端上架商品1个；H5与小程序使用同一账号；商品/SKU/库存/价格初始值已记录</x:v>
+        <x:v>不同用户A/B及各自地址；同一可售SKU库存=1；各自购物车数量=1；记录原库存；使用同步屏障同时提交</x:v>
       </x:c>
       <x:c r="H6" s="53" t="str">
         <x:v>至多一个订单成功；失败方明确；数据库库存非负</x:v>
@@ -7419,7 +7437,7 @@
         <x:v>两侧均为取消；后台不能再受理/退款</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="48" customHeight="1">
+    <x:row r="18" ht="24" hidden="0" customHeight="1">
       <x:c r="A18" s="50" t="str">
         <x:v>E2E-017</x:v>
       </x:c>
@@ -7440,7 +7458,7 @@
 2. B 参团支付</x:v>
       </x:c>
       <x:c r="G18" s="51" t="str">
-        <x:v>用户A；有效商品/SKU；地址；优惠券；待付款至已完成订单状态数据</x:v>
+        <x:v>不同用户A/B及各自地址；人数=2的有效团购规则；足够库存；已配置支付沙箱或合法Mock回调</x:v>
       </x:c>
       <x:c r="H18" s="53" t="str">
         <x:v>两订单和团成员关联正确；达到人数后团状态成功</x:v>
@@ -7555,7 +7573,7 @@
         <x:v>用户端读取新值；重启后仍保存；无缓存长期不一致</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" ht="48" customHeight="1">
+    <x:row r="23" ht="24" hidden="0" customHeight="1">
       <x:c r="A23" s="50" t="str">
         <x:v>E2E-022</x:v>
       </x:c>
@@ -7576,13 +7594,13 @@
 2. 尝试查看、创建、删除商品及直接调用 API</x:v>
       </x:c>
       <x:c r="G23" s="51" t="str">
-        <x:v>管理端上架商品1个；H5与小程序使用同一账号；商品/SKU/库存/价格初始值已记录</x:v>
+        <x:v>超级管理员及独立的只读管理员；只读角色仅授予商品查看权限；准备商品ID与创建、删除接口；保存角色原权限</x:v>
       </x:c>
       <x:c r="H23" s="53" t="str">
         <x:v>只能查看；创建删除菜单和服务端均拒绝；操作日志可追踪</x:v>
       </x:c>
     </x:row>
-    <x:row r="24" ht="48" customHeight="1">
+    <x:row r="24" ht="190" hidden="0" customHeight="1">
       <x:c r="A24" s="50" t="str">
         <x:v>E2E-023</x:v>
       </x:c>
@@ -7599,11 +7617,14 @@
         <x:v>后端、MySQL及涉及的客户端/管理端可访问；用户 A/B 均有地址、购物车、订单、售后</x:v>
       </x:c>
       <x:c r="F24" s="51" t="str">
-        <x:v>1. B 使用 A 的各类 ID 构造请求
-2. 观察页面提示、接口响应及业务状态</x:v>
+        <x:v>1. 以用户A创建地址、购物车及订单等资源并保存ID
+2. 用A身份验证合法访问作为基线
+3. 切换为B的Token，保持A的对象ID不变，逐项查询、修改、删除或提交
+4. 组合B地址与A购物车提交订单，核对响应、订单归属、A购物车和库存
+5. 保存越权结果证据，清理仅由本次测试创建的数据</x:v>
       </x:c>
       <x:c r="G24" s="51" t="str">
-        <x:v>用户A；有效商品/SKU；地址；优惠券；待付款至已完成订单状态数据</x:v>
+        <x:v>不同用户A/B及各自Token；A的addressId、cartId、orderId及售后ID；B的有效地址；记录A对象归属和数据库状态</x:v>
       </x:c>
       <x:c r="H24" s="53" t="str">
         <x:v>地址/购物车/订单/评价/售后全部拒绝；A 数据不变</x:v>

</xml_diff>